<commit_message>
Fix typo in file
</commit_message>
<xml_diff>
--- a/datascience/suitability_scoring/notebooks/temp_data/species.xlsx
+++ b/datascience/suitability_scoring/notebooks/temp_data/species.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\darrin\Work\Planting_Optimisation_tool_dws\datascience\suitability_scoring\notebooks\temp_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB5A73E9-98C4-4B4D-A6AD-B24DB43DE655}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B99664C9-2281-4197-B2AF-AE2A912ECFB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="57480" yWindow="-285" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="78">
   <si>
     <t>Casuarina equisetifolia</t>
   </si>
@@ -233,9 +233,6 @@
   </si>
   <si>
     <t>Ai-silose/Copperpod</t>
-  </si>
-  <si>
-    <t>FLASE</t>
   </si>
   <si>
     <t>block, boundary</t>
@@ -684,7 +681,7 @@
         <v>1</v>
       </c>
       <c r="R2" s="5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="3" spans="1:18" ht="12.5" x14ac:dyDescent="0.25">
@@ -740,7 +737,7 @@
         <v>1</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="4" spans="1:18" ht="12.5" x14ac:dyDescent="0.25">
@@ -796,7 +793,7 @@
         <v>1</v>
       </c>
       <c r="R4" s="5" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="5" spans="1:18" ht="25" x14ac:dyDescent="0.25">
@@ -852,7 +849,7 @@
         <v>0</v>
       </c>
       <c r="R5" s="5" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="6" spans="1:18" ht="25" x14ac:dyDescent="0.25">
@@ -908,7 +905,7 @@
         <v>1</v>
       </c>
       <c r="R6" s="6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="7" spans="1:18" ht="25" x14ac:dyDescent="0.25">
@@ -964,7 +961,7 @@
         <v>1</v>
       </c>
       <c r="R7" s="6" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="8" spans="1:18" ht="25" x14ac:dyDescent="0.25">
@@ -1020,7 +1017,7 @@
         <v>1</v>
       </c>
       <c r="R8" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="9" spans="1:18" ht="25" x14ac:dyDescent="0.25">
@@ -1076,7 +1073,7 @@
         <v>1</v>
       </c>
       <c r="R9" s="6" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="10" spans="1:18" ht="25" x14ac:dyDescent="0.25">
@@ -1132,7 +1129,7 @@
         <v>0</v>
       </c>
       <c r="R10" s="5" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="11" spans="1:18" ht="12.5" x14ac:dyDescent="0.25">
@@ -1188,7 +1185,7 @@
         <v>1</v>
       </c>
       <c r="R11" s="6" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="12" spans="1:18" ht="25" x14ac:dyDescent="0.25">
@@ -1244,7 +1241,7 @@
         <v>0</v>
       </c>
       <c r="R12" s="5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="13" spans="1:18" ht="25" x14ac:dyDescent="0.25">
@@ -1300,7 +1297,7 @@
         <v>1</v>
       </c>
       <c r="R13" s="5" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="14" spans="1:18" ht="12.5" x14ac:dyDescent="0.25">
@@ -1356,7 +1353,7 @@
         <v>0</v>
       </c>
       <c r="R14" s="5" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="15" spans="1:18" ht="12.5" x14ac:dyDescent="0.25">
@@ -1412,7 +1409,7 @@
         <v>1</v>
       </c>
       <c r="R15" s="6" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="16" spans="1:18" ht="12.5" x14ac:dyDescent="0.25">
@@ -1468,7 +1465,7 @@
         <v>1</v>
       </c>
       <c r="R16" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="17" spans="1:19" ht="75" x14ac:dyDescent="0.25">
@@ -1524,7 +1521,7 @@
         <v>0</v>
       </c>
       <c r="R17" s="5" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="18" spans="1:19" ht="37.5" x14ac:dyDescent="0.25">
@@ -1580,7 +1577,7 @@
         <v>0</v>
       </c>
       <c r="R18" s="5" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="19" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1623,20 +1620,20 @@
       <c r="M19" s="6" t="b">
         <v>0</v>
       </c>
-      <c r="N19" s="6" t="s">
+      <c r="N19" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="O19" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="P19" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q19" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="R19" s="6" t="s">
         <v>71</v>
-      </c>
-      <c r="O19" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="P19" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q19" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="R19" s="6" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="20" spans="1:19" ht="37.5" x14ac:dyDescent="0.25">
@@ -1692,7 +1689,7 @@
         <v>0</v>
       </c>
       <c r="R20" s="7" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="S20" s="2"/>
     </row>
@@ -1749,7 +1746,7 @@
         <v>0</v>
       </c>
       <c r="R21" s="7" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="S21" s="1"/>
     </row>
@@ -1776,15 +1773,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100364D73228578DF4DB485C574B69A0DE9" ma:contentTypeVersion="22" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="52a3386525053e6db11b716e7def64b9">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5433951f-06c3-4618-8b57-3de8e57a9660" xmlns:ns3="7998ff36-f67b-497d-9ba5-0737ce74e881" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="bdd95e8bdbb8a6e33b28404e6fa50ffb" ns2:_="" ns3:_="">
     <xsd:import namespace="5433951f-06c3-4618-8b57-3de8e57a9660"/>
@@ -2072,6 +2060,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0D1BA54D-BC7F-4C87-BE46-2D5F9FE86096}">
   <ds:schemaRefs>
@@ -2084,14 +2081,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3CDE8AF1-C67E-44CB-ADB2-0710A241AF03}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4D1DD424-7DAD-4DB2-A539-D30B372CDB8E}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2108,4 +2097,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3CDE8AF1-C67E-44CB-ADB2-0710A241AF03}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Fix type in species file
</commit_message>
<xml_diff>
--- a/datascience/suitability_scoring/notebooks/temp_data/species.xlsx
+++ b/datascience/suitability_scoring/notebooks/temp_data/species.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\darrin\Work\Planting_Optimisation_tool_dws\datascience\suitability_scoring\notebooks\temp_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB5A73E9-98C4-4B4D-A6AD-B24DB43DE655}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DCCF094-CF4B-49F2-A341-DB2C14F6D1E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="57480" yWindow="-285" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="78">
   <si>
     <t>Casuarina equisetifolia</t>
   </si>
@@ -233,9 +233,6 @@
   </si>
   <si>
     <t>Ai-silose/Copperpod</t>
-  </si>
-  <si>
-    <t>FLASE</t>
   </si>
   <si>
     <t>block, boundary</t>
@@ -684,7 +681,7 @@
         <v>1</v>
       </c>
       <c r="R2" s="5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="3" spans="1:18" ht="12.5" x14ac:dyDescent="0.25">
@@ -740,7 +737,7 @@
         <v>1</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="4" spans="1:18" ht="12.5" x14ac:dyDescent="0.25">
@@ -796,7 +793,7 @@
         <v>1</v>
       </c>
       <c r="R4" s="5" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="5" spans="1:18" ht="25" x14ac:dyDescent="0.25">
@@ -852,7 +849,7 @@
         <v>0</v>
       </c>
       <c r="R5" s="5" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="6" spans="1:18" ht="25" x14ac:dyDescent="0.25">
@@ -908,7 +905,7 @@
         <v>1</v>
       </c>
       <c r="R6" s="6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="7" spans="1:18" ht="25" x14ac:dyDescent="0.25">
@@ -964,7 +961,7 @@
         <v>1</v>
       </c>
       <c r="R7" s="6" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="8" spans="1:18" ht="25" x14ac:dyDescent="0.25">
@@ -1020,7 +1017,7 @@
         <v>1</v>
       </c>
       <c r="R8" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="9" spans="1:18" ht="25" x14ac:dyDescent="0.25">
@@ -1076,7 +1073,7 @@
         <v>1</v>
       </c>
       <c r="R9" s="6" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="10" spans="1:18" ht="25" x14ac:dyDescent="0.25">
@@ -1132,7 +1129,7 @@
         <v>0</v>
       </c>
       <c r="R10" s="5" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="11" spans="1:18" ht="12.5" x14ac:dyDescent="0.25">
@@ -1188,7 +1185,7 @@
         <v>1</v>
       </c>
       <c r="R11" s="6" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="12" spans="1:18" ht="25" x14ac:dyDescent="0.25">
@@ -1244,7 +1241,7 @@
         <v>0</v>
       </c>
       <c r="R12" s="5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="13" spans="1:18" ht="25" x14ac:dyDescent="0.25">
@@ -1300,7 +1297,7 @@
         <v>1</v>
       </c>
       <c r="R13" s="5" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="14" spans="1:18" ht="12.5" x14ac:dyDescent="0.25">
@@ -1356,7 +1353,7 @@
         <v>0</v>
       </c>
       <c r="R14" s="5" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="15" spans="1:18" ht="12.5" x14ac:dyDescent="0.25">
@@ -1412,7 +1409,7 @@
         <v>1</v>
       </c>
       <c r="R15" s="6" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="16" spans="1:18" ht="12.5" x14ac:dyDescent="0.25">
@@ -1468,7 +1465,7 @@
         <v>1</v>
       </c>
       <c r="R16" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="17" spans="1:19" ht="75" x14ac:dyDescent="0.25">
@@ -1524,7 +1521,7 @@
         <v>0</v>
       </c>
       <c r="R17" s="5" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="18" spans="1:19" ht="37.5" x14ac:dyDescent="0.25">
@@ -1580,7 +1577,7 @@
         <v>0</v>
       </c>
       <c r="R18" s="5" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="19" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1623,20 +1620,20 @@
       <c r="M19" s="6" t="b">
         <v>0</v>
       </c>
-      <c r="N19" s="6" t="s">
+      <c r="N19" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="O19" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="P19" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q19" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="R19" s="6" t="s">
         <v>71</v>
-      </c>
-      <c r="O19" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="P19" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q19" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="R19" s="6" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="20" spans="1:19" ht="37.5" x14ac:dyDescent="0.25">
@@ -1692,7 +1689,7 @@
         <v>0</v>
       </c>
       <c r="R20" s="7" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="S20" s="2"/>
     </row>
@@ -1749,7 +1746,7 @@
         <v>0</v>
       </c>
       <c r="R21" s="7" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="S21" s="1"/>
     </row>
@@ -1776,15 +1773,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100364D73228578DF4DB485C574B69A0DE9" ma:contentTypeVersion="22" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="52a3386525053e6db11b716e7def64b9">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5433951f-06c3-4618-8b57-3de8e57a9660" xmlns:ns3="7998ff36-f67b-497d-9ba5-0737ce74e881" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="bdd95e8bdbb8a6e33b28404e6fa50ffb" ns2:_="" ns3:_="">
     <xsd:import namespace="5433951f-06c3-4618-8b57-3de8e57a9660"/>
@@ -2072,6 +2060,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0D1BA54D-BC7F-4C87-BE46-2D5F9FE86096}">
   <ds:schemaRefs>
@@ -2084,14 +2081,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3CDE8AF1-C67E-44CB-ADB2-0710A241AF03}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4D1DD424-7DAD-4DB2-A539-D30B372CDB8E}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2108,4 +2097,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3CDE8AF1-C67E-44CB-ADB2-0710A241AF03}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>